<commit_message>
committed @ 2025-10-13-091911-0500 by tcn85@rtsjpl774kw20.managed.mst.edu
</commit_message>
<xml_diff>
--- a/data/3420-2025-fall-quizzes/3420-2025-fall-py-review-01.xlsx
+++ b/data/3420-2025-fall-quizzes/3420-2025-fall-py-review-01.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tcn85/workspace/dsm/data/3420-2025-fall-quizzes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E51DFCBB-1911-F948-9780-01F738FB4D71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8506346C-B3BB-1448-B661-87F5CB10DA1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29860" yWindow="680" windowWidth="10820" windowHeight="13260" xr2:uid="{02943BD8-8D23-1D42-A928-8937731C9A90}"/>
+    <workbookView xWindow="-18160" yWindow="4220" windowWidth="17200" windowHeight="13260" xr2:uid="{02943BD8-8D23-1D42-A928-8937731C9A90}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="py-np-pd" sheetId="2" r:id="rId1"/>
+    <sheet name="py-review" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="31">
   <si>
     <t>name</t>
   </si>
@@ -170,78 +171,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -570,9 +500,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{253F1E1C-F588-7C4E-B050-53E91BB391E3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72BE9F46-4462-794B-8946-25A04D6D2C07}">
   <dimension ref="A1:L20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
     <col min="2" max="10" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -621,6 +551,154 @@
       <c r="A2" t="s">
         <v>20</v>
       </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{253F1E1C-F588-7C4E-B050-53E91BB391E3}">
+  <dimension ref="A1:L20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="10" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="5.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
       <c r="B2">
         <v>1</v>
       </c>

</xml_diff>